<commit_message>
fix(tarea_2): protege datos personales publicados
</commit_message>
<xml_diff>
--- a/tarea_2/auditoria_humana.xlsx
+++ b/tarea_2/auditoria_humana.xlsx
@@ -350,14 +350,13 @@
     <t xml:space="preserve">CEPIANK
 Centro Nacicnal de Plancamiento Estizégico
 Firmado digitalmente por
-VALCARCEL SALDAÑA Juan Julio
+[PERSONA_20]
 FAU 20520594451 soft
 Motivo: Doy Vv° B
 Fecha: 26.05.2026 15:48:47 -05:00
 CEPLAAK
 Centro Nacicnal de Plancamiento Estrzógico
-Firmado digitalmente por MORI
-KURIYAMA Virgilio Antonio FAU
+Firmado digitalmente por [PERSONA_21] FAU
 20520594451 soft
 Motivo: Doy V° B°
 Fecha: 26.05.2026 15:53:17 -05:00
@@ -367,8 +366,7 @@
 formalización mediante Resolución de Presidencia del Consejo Directivo, por encontrarse
 Centro Nacicnal de Plancamiento Estizégico
 alineada con el marco normativo vigente y los objetivos institucionales del CEPLAN;
-Firmado digitalmente por DE LA
-FLOR SAENZ Luis Enrique FAU
+Firmado digitalmente por [PERSONA_22] FAU
 20520594451 soft
 Motivo: Doy V° B°
 Con el visado del Director Ejecutivo, del Jefe de la Oficina de Planeamiento y
@@ -464,7 +462,7 @@
     <t>{
  "modalidad": "audio",
  "tema": "Entrevista sobre percepción del Perú",
- "resumen": "Jean‑Pierre Venegas, estudiante de la Universidad Nacional Mayor de San Marcos, habla sobre los aspectos positivos y negativos del Perú y da consejos a los jóvenes, enfatizando la educación, el ahorro y la prudencia financiera.",
+ "resumen": "[PERSONA_6], estudiante de la Universidad Nacional Mayor de San Marcos, habla sobre los aspectos positivos y negativos del Perú y da consejos a los jóvenes, enfatizando la educación, el ahorro y la prudencia financiera.",
  "citas_clave": [
   "Perú es un país con mucha historia, el lugar donde yo nací, y me gusta.",
   "No preste dinero, no seas a valde nadie, y ahorra tu dinero.",
@@ -474,7 +472,7 @@
 }</t>
   </si>
   <si>
-    <t>[00:00:00] A ver, buenas noches, primeramente es mi nombre Jean-Piervenegas, soy estudiante de la Universidad San Marcos. A ver un momento, por favor. Yo te voy a decir la verdad. Sí, no, está bien, es lo que yo busco. A ver, buenas noches. Si, buenas noches, mi nombre es Jean-Pierre Venegas, soy estudiante de la Universidad San Marcos. ¿Cómo se llama usted? Alex Giles. Señor Alex, esta entrevista va a ser publicada en un foro de internet, ¿está de acuerdo? Exacto, sí. Muy bien, ¿qué es el Perú para usted? Perú es un país con mucha historia, bueno, el lugar donde yo nací, y me gusta. ¿Cuáles serían los principales aspectos positivos que rescata el Perú? Mira, realmente. en el Perú, aunque tengas problemas, ya sea del poder judicial o de todo el sistema en sí, yo pienso que para mí lo beneficioso de este país es la enseñanza que nos da cómo ganarnos el dinero. Porque como yo lo veo, este es un país, créanme, muy rico, que yo no sé cómo hace la gente, pero aquí la gente tiene dinero, pero no lo sabe cómo realmente ahorrarlo o conservarlo, ¿me entiendes? Lo donde yo vengo, crees, me tengo que venir acá a inspirarme, para llevarme lo que yo veo aquí. para poder ganarme todo el dinero q</t>
+    <t>[00:00:00] A ver, buenas noches, primeramente es mi nombre [PERSONA_6], soy estudiante de la Universidad San Marcos. A ver un momento, por favor. Yo te voy a decir la verdad. Sí, no, está bien, es lo que yo busco. A ver, buenas noches. Si, buenas noches, mi nombre es [PERSONA_6], soy estudiante de la Universidad San Marcos. ¿Cómo se llama usted? [PERSONA_7]. Señor [PERSONA_7], esta entrevista va a ser publicada en un foro de internet, ¿está de acuerdo? Exacto, sí. Muy bien, ¿qué es el Perú para usted? Perú es un país con mucha historia, bueno, el lugar donde yo nací, y me gusta. ¿Cuáles serían los principales aspectos positivos que rescata el Perú? Mira, realmente. en el Perú, aunque tengas problemas, ya sea del poder judicial o de todo el sistema en sí, yo pienso que para mí lo beneficioso de este país es la enseñanza que nos da cómo ganarnos el dinero. Porque como yo lo veo, este es un país, créanme, muy rico, que yo no sé cómo hace la gente, pero aquí la gente tiene dinero, pero no lo sabe cómo realmente ahorrarlo o conservarlo, ¿me entiendes? Lo donde yo vengo, crees, me tengo que venir acá a inspirarme, para llevarme lo que yo veo aquí. para poder ganarme todo el dinero q</t>
   </si>
   <si>
     <t>clip_24</t>
@@ -540,7 +538,7 @@
     <t>{
  "modalidad": "audio",
  "tema": "Significado del Perú y sus características",
- "resumen": "En la entrevista Carlos Ramírez reflexiona sobre el significado del Perú como la tierra que acoge a sus habitantes y menciona tanto aspectos positivos como el avance gradual, como negativos la corrupción y malas funciones de las autoridades.",
+ "resumen": "En la entrevista [PERSONA_8] reflexiona sobre el significado del Perú como la tierra que acoge a sus habitantes y menciona tanto aspectos positivos como el avance gradual, como negativos la corrupción y malas funciones de las autoridades.",
  "citas_clave": [
   "el Perú debe significar casi todo porque es la tierra donde estamos",
   "Las malas funciones que hacen nuestras autoridades",
@@ -550,7 +548,7 @@
 }</t>
   </si>
   <si>
-    <t>[00:00:00] Nos encontramos aquí con el señor Carlos Ramírez, señor Carlos, esta entrevista va a ser subida en internet, ¿está usted de acuerdo con eso? Sí, muchas gracias. La primera pregunta es ¿Qué significa el Perú para usted? ¿Qué significa el Perú? Yo pienso que para cada Perú el Perú debe significar casi todo porque es la tierra donde estamos. Si lo vemos en aspecto geográfico, ¿no? En lo cual, a pesar de nuestras descendencias, de todas nuestras descendencias es la tierra que nos acoge, ¿no? Que es ese límite que se llama Perú. ¿En el Perú cuáles serían las características positivas más resaltantes que usted puede notar? Las características que cada vez vamos avanzando de a poco, ¿no? Subtítulos por la comunidad de Amara.org como por ejemplo que no podemos comparar la época del birreinato con la actualidad cada momento va avanzando, son caracterices que vas, como te puedo decir, que vas desarrollando ¿Y cuáles serían las características negativas que usted puede observar? Indudablemente el... Las malas funciones que hacen nuestras autoridades, si veremos en el lado político, la corrupción... Muchas gracias, señor. Feliz de fiestas, padre.</t>
+    <t>[00:00:00] Nos encontramos aquí con el señor [PERSONA_8], señor [PERSONA_8], esta entrevista va a ser subida en internet, ¿está usted de acuerdo con eso? Sí, muchas gracias. La primera pregunta es ¿Qué significa el Perú para usted? ¿Qué significa el Perú? Yo pienso que para cada Perú el Perú debe significar casi todo porque es la tierra donde estamos. Si lo vemos en aspecto geográfico, ¿no? En lo cual, a pesar de nuestras descendencias, de todas nuestras descendencias es la tierra que nos acoge, ¿no? Que es ese límite que se llama Perú. ¿En el Perú cuáles serían las características positivas más resaltantes que usted puede notar? Las características que cada vez vamos avanzando de a poco, ¿no? Subtítulos por la comunidad de Amara.org como por ejemplo que no podemos comparar la época del birreinato con la actualidad cada momento va avanzando, son caracterices que vas, como te puedo decir, que vas desarrollando ¿Y cuáles serían las características negativas que usted puede observar? Indudablemente el... Las malas funciones que hacen nuestras autoridades, si veremos en el lado político, la corrupción... Muchas gracias, señor. Feliz de fiestas, padre.</t>
   </si>
   <si>
     <t>clip_10_d</t>

</xml_diff>